<commit_message>
Improving format for benchmark comparison template
</commit_message>
<xml_diff>
--- a/src/modules/reports/report-templates/benchmark-comparison.xlsx
+++ b/src/modules/reports/report-templates/benchmark-comparison.xlsx
@@ -2527,7 +2527,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2536,17 +2536,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF162630"/>
+        <fgColor rgb="FF2E1065"/>
+        <bgColor rgb="FF2E1065"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2403B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA9AAAD"/>
+        <fgColor rgb="FFE2E8F0"/>
+        <bgColor rgb="FFE2E8F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -2571,16 +2568,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2980,7 +2977,7 @@
     <col min="2" max="9" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3004,7 +3001,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" ht="21.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" ht="27" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
@@ -3023,7 +3020,7 @@
       </c>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" ht="19.95" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" ht="24.95" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -3042,7 +3039,7 @@
       </c>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" ht="27" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" ht="33.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="3" t="s">
         <v>6</v>
@@ -3061,7 +3058,7 @@
       </c>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" ht="40.05" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" ht="50.1" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -3114,7 +3111,7 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -3143,7 +3140,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -3172,7 +3169,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -3201,7 +3198,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -3230,7 +3227,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>56</v>
       </c>
@@ -3259,7 +3256,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -3288,7 +3285,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -3317,7 +3314,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>83</v>
       </c>
@@ -3346,7 +3343,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>92</v>
       </c>
@@ -3375,7 +3372,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>101</v>
       </c>
@@ -3417,7 +3414,7 @@
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
     </row>
-    <row r="20" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>111</v>
       </c>
@@ -3446,7 +3443,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>120</v>
       </c>
@@ -3475,7 +3472,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="22" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>129</v>
       </c>
@@ -3504,7 +3501,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="23" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>138</v>
       </c>
@@ -3533,7 +3530,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="24" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>147</v>
       </c>
@@ -3562,7 +3559,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="25" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>156</v>
       </c>
@@ -3591,7 +3588,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="26" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>165</v>
       </c>
@@ -3620,7 +3617,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="27" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>174</v>
       </c>
@@ -3649,7 +3646,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="28" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>183</v>
       </c>
@@ -3678,7 +3675,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="29" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>192</v>
       </c>
@@ -3707,7 +3704,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="30" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>201</v>
       </c>
@@ -3736,7 +3733,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="31" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>210</v>
       </c>
@@ -3765,7 +3762,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="32" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>219</v>
       </c>
@@ -3807,7 +3804,7 @@
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
     </row>
-    <row r="34" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>229</v>
       </c>
@@ -3836,7 +3833,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="35" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>238</v>
       </c>
@@ -3865,7 +3862,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="36" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>247</v>
       </c>
@@ -3894,7 +3891,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="37" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>256</v>
       </c>
@@ -3923,7 +3920,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="38" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>265</v>
       </c>
@@ -3952,7 +3949,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="39" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>274</v>
       </c>
@@ -3981,7 +3978,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="40" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>283</v>
       </c>
@@ -4010,7 +4007,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="41" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>292</v>
       </c>
@@ -4039,7 +4036,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="42" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>301</v>
       </c>
@@ -4068,7 +4065,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="43" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>310</v>
       </c>
@@ -4097,7 +4094,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="44" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>319</v>
       </c>
@@ -4126,7 +4123,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="45" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>328</v>
       </c>
@@ -4168,7 +4165,7 @@
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
     </row>
-    <row r="47" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>338</v>
       </c>
@@ -4197,7 +4194,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="48" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>347</v>
       </c>
@@ -4226,7 +4223,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="49" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>356</v>
       </c>
@@ -4255,7 +4252,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="50" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>365</v>
       </c>
@@ -4284,7 +4281,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="51" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>374</v>
       </c>
@@ -4313,7 +4310,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="52" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>383</v>
       </c>
@@ -4342,7 +4339,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="53" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>392</v>
       </c>
@@ -4371,7 +4368,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="54" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>401</v>
       </c>
@@ -4400,7 +4397,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="55" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>410</v>
       </c>
@@ -4429,7 +4426,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="56" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>419</v>
       </c>
@@ -4471,7 +4468,7 @@
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
     </row>
-    <row r="58" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>429</v>
       </c>
@@ -4500,7 +4497,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="59" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>438</v>
       </c>
@@ -4529,7 +4526,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="60" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>447</v>
       </c>
@@ -4558,7 +4555,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="61" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>456</v>
       </c>
@@ -4587,7 +4584,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="62" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>465</v>
       </c>
@@ -4616,7 +4613,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="63" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>474</v>
       </c>
@@ -4645,7 +4642,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="64" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>483</v>
       </c>
@@ -4674,7 +4671,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="65" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>492</v>
       </c>
@@ -4716,7 +4713,7 @@
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
     </row>
-    <row r="67" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>502</v>
       </c>
@@ -4745,7 +4742,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="68" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>511</v>
       </c>
@@ -4774,7 +4771,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="69" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>520</v>
       </c>
@@ -4803,7 +4800,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="70" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>529</v>
       </c>
@@ -4832,7 +4829,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="71" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>538</v>
       </c>
@@ -4861,7 +4858,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="72" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>547</v>
       </c>
@@ -4890,7 +4887,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="73" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>556</v>
       </c>
@@ -4932,7 +4929,7 @@
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
     </row>
-    <row r="75" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>566</v>
       </c>
@@ -4961,7 +4958,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="76" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>575</v>
       </c>
@@ -4990,7 +4987,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="77" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>584</v>
       </c>
@@ -5019,7 +5016,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="78" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>593</v>
       </c>
@@ -5048,7 +5045,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="79" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>602</v>
       </c>
@@ -5077,7 +5074,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="80" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>611</v>
       </c>
@@ -5119,7 +5116,7 @@
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
     </row>
-    <row r="82" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>621</v>
       </c>
@@ -5148,7 +5145,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="83" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>630</v>
       </c>
@@ -5177,7 +5174,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="84" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>639</v>
       </c>
@@ -5206,7 +5203,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="85" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>648</v>
       </c>
@@ -5235,7 +5232,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="86" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>657</v>
       </c>
@@ -5264,7 +5261,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="87" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>666</v>
       </c>
@@ -5293,7 +5290,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="88" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>675</v>
       </c>
@@ -5322,7 +5319,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="89" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>684</v>
       </c>
@@ -5351,7 +5348,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="90" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>693</v>
       </c>
@@ -5380,7 +5377,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="91" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>702</v>
       </c>
@@ -5409,7 +5406,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="92" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>711</v>
       </c>
@@ -5438,7 +5435,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="93" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>720</v>
       </c>
@@ -5467,7 +5464,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="94" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>729</v>
       </c>
@@ -5496,7 +5493,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="95" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>738</v>
       </c>
@@ -5538,7 +5535,7 @@
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
     </row>
-    <row r="97" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>748</v>
       </c>
@@ -5567,7 +5564,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="98" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>757</v>
       </c>
@@ -5596,7 +5593,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="99" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>766</v>
       </c>
@@ -5625,7 +5622,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="100" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>775</v>
       </c>
@@ -5654,7 +5651,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="101" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>784</v>
       </c>
@@ -5683,7 +5680,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="102" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>793</v>
       </c>
@@ -5712,7 +5709,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="103" ht="15.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
         <v>802</v>
       </c>
@@ -5741,7 +5738,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="104" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" ht="18.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
         <v>811</v>
       </c>
@@ -5770,7 +5767,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="105" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" ht="18.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
         <v>820</v>
       </c>
@@ -5783,7 +5780,7 @@
       <c r="H105" s="10"/>
       <c r="I105" s="10"/>
     </row>
-    <row r="106" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" ht="18.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
         <v>821</v>
       </c>

</xml_diff>